<commit_message>
feat: Complete application development and documentation
- Add all application features and components
- Include frontend and backend implementations
- Add workflow engine and module parameter systems
- Add import/export functionality for hardware configs
- Include comprehensive documentation and guides
- Add test files and sample data
- Update .gitignore to exclude Windows reserved filenames
</commit_message>
<xml_diff>
--- a/Sample_HW_IOList_AS01.xlsx
+++ b/Sample_HW_IOList_AS01.xlsx
@@ -1,18 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0157AC7-10C5-4E52-918D-7068D553B5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="HW_IO_List" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Info" state="visible" r:id="rId5"/>
+    <sheet name="HW_IO_List" sheetId="1" r:id="rId1"/>
+    <sheet name="Info" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="112">
   <si>
     <t>Subsystem_No</t>
   </si>
@@ -140,144 +158,36 @@
     <t>DI16 x 24VDC ST V0.0</t>
   </si>
   <si>
-    <t>101-XS-001</t>
-  </si>
-  <si>
     <t>Valve 1 Open Limit</t>
   </si>
   <si>
     <t>DI</t>
   </si>
   <si>
-    <t>101-XS-002</t>
-  </si>
-  <si>
     <t>Valve 1 Closed Limit</t>
   </si>
   <si>
-    <t>101-XS-003</t>
-  </si>
-  <si>
     <t>Valve 2 Open Limit</t>
   </si>
   <si>
-    <t>101-XS-004</t>
-  </si>
-  <si>
     <t>Valve 2 Closed Limit</t>
   </si>
   <si>
-    <t>101-XS-005</t>
-  </si>
-  <si>
-    <t>Pump 1 Running</t>
-  </si>
-  <si>
-    <t>101-XS-006</t>
-  </si>
-  <si>
-    <t>Pump 1 Fault</t>
-  </si>
-  <si>
-    <t>101-XS-007</t>
-  </si>
-  <si>
-    <t>Pump 2 Running</t>
-  </si>
-  <si>
-    <t>101-XS-008</t>
-  </si>
-  <si>
-    <t>Pump 2 Fault</t>
-  </si>
-  <si>
-    <t>101-XS-009</t>
-  </si>
-  <si>
-    <t>Level High High</t>
-  </si>
-  <si>
-    <t>101-XS-010</t>
-  </si>
-  <si>
-    <t>Level High</t>
-  </si>
-  <si>
-    <t>101-XS-011</t>
-  </si>
-  <si>
-    <t>Level Low</t>
-  </si>
-  <si>
-    <t>101-XS-012</t>
-  </si>
-  <si>
-    <t>Level Low Low</t>
-  </si>
-  <si>
-    <t>101-XS-013</t>
-  </si>
-  <si>
-    <t>Emergency Stop</t>
-  </si>
-  <si>
-    <t>101-XS-014</t>
-  </si>
-  <si>
-    <t>Fire Alarm</t>
-  </si>
-  <si>
-    <t>101-XS-015</t>
-  </si>
-  <si>
-    <t>Gas Detector 1</t>
-  </si>
-  <si>
-    <t>101-XS-016</t>
-  </si>
-  <si>
-    <t>Gas Detector 2</t>
-  </si>
-  <si>
     <t>6ES7 132-6BH01-0BA0</t>
   </si>
   <si>
     <t>DQ16 x 24VDC/0.5A ST V0~</t>
   </si>
   <si>
-    <t>101-YC-001</t>
-  </si>
-  <si>
     <t>Valve 1 Open Command</t>
   </si>
   <si>
     <t>DO</t>
   </si>
   <si>
-    <t>101-YC-002</t>
-  </si>
-  <si>
-    <t>Valve 1 Close Command</t>
-  </si>
-  <si>
-    <t>101-YC-003</t>
-  </si>
-  <si>
     <t>Valve 2 Open Command</t>
   </si>
   <si>
-    <t>101-YC-004</t>
-  </si>
-  <si>
-    <t>Valve 2 Close Command</t>
-  </si>
-  <si>
-    <t>101-YC-005</t>
-  </si>
-  <si>
-    <t>Pump 1 Start</t>
-  </si>
-  <si>
     <t>101-YC-006</t>
   </si>
   <si>
@@ -384,22 +294,96 @@
   </si>
   <si>
     <t>Channel number within the module, 0-based (empty for INFRA)</t>
+  </si>
+  <si>
+    <t>XV001_GSH</t>
+  </si>
+  <si>
+    <t>XV002_GSH</t>
+  </si>
+  <si>
+    <t>XV003_GSH</t>
+  </si>
+  <si>
+    <t>XV004_GSH</t>
+  </si>
+  <si>
+    <t>XV005_GSH</t>
+  </si>
+  <si>
+    <t>XV001_GSL</t>
+  </si>
+  <si>
+    <t>XV002_GSL</t>
+  </si>
+  <si>
+    <t>XV003_GSL</t>
+  </si>
+  <si>
+    <t>XV004_GSL</t>
+  </si>
+  <si>
+    <t>XV005_GSL</t>
+  </si>
+  <si>
+    <t>XV001_OUT</t>
+  </si>
+  <si>
+    <t>XV002_OUT</t>
+  </si>
+  <si>
+    <t>XV003_OUT</t>
+  </si>
+  <si>
+    <t>XV004_OUT</t>
+  </si>
+  <si>
+    <t>XV005_OUT</t>
+  </si>
+  <si>
+    <t>Valve 3 Open Limit</t>
+  </si>
+  <si>
+    <t>Valve 3 Closed Limit</t>
+  </si>
+  <si>
+    <t>Valve 4 Open Limit</t>
+  </si>
+  <si>
+    <t>Valve 4 Closed Limit</t>
+  </si>
+  <si>
+    <t>Valve 5 Open Limit</t>
+  </si>
+  <si>
+    <t>Valve 5 Closed Limit</t>
+  </si>
+  <si>
+    <t>Valve 3 Open Command</t>
+  </si>
+  <si>
+    <t>Valve 4 Open Command</t>
+  </si>
+  <si>
+    <t>Valve 5 Open Command</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -769,20 +753,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L43"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="32" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="32.7109375" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1165,13 +1149,13 @@
         <v>41</v>
       </c>
       <c r="I11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" t="s">
         <v>42</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>43</v>
-      </c>
-      <c r="K11" t="s">
-        <v>44</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1200,13 +1184,13 @@
         <v>41</v>
       </c>
       <c r="I12" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="J12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L12">
         <v>1</v>
@@ -1235,13 +1219,13 @@
         <v>41</v>
       </c>
       <c r="I13" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="J13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="K13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L13">
         <v>2</v>
@@ -1270,13 +1254,13 @@
         <v>41</v>
       </c>
       <c r="I14" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="J14" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="K14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L14">
         <v>3</v>
@@ -1305,13 +1289,13 @@
         <v>41</v>
       </c>
       <c r="I15" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="J15" t="s">
-        <v>52</v>
+        <v>103</v>
       </c>
       <c r="K15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L15">
         <v>4</v>
@@ -1340,13 +1324,13 @@
         <v>41</v>
       </c>
       <c r="I16" t="s">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="J16" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="K16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -1375,13 +1359,13 @@
         <v>41</v>
       </c>
       <c r="I17" t="s">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="J17" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="K17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L17">
         <v>6</v>
@@ -1410,13 +1394,13 @@
         <v>41</v>
       </c>
       <c r="I18" t="s">
-        <v>57</v>
+        <v>96</v>
       </c>
       <c r="J18" t="s">
-        <v>58</v>
+        <v>106</v>
       </c>
       <c r="K18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L18">
         <v>7</v>
@@ -1445,13 +1429,13 @@
         <v>41</v>
       </c>
       <c r="I19" t="s">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="J19" t="s">
-        <v>60</v>
+        <v>107</v>
       </c>
       <c r="K19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L19">
         <v>8</v>
@@ -1480,13 +1464,13 @@
         <v>41</v>
       </c>
       <c r="I20" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
       <c r="J20" t="s">
-        <v>62</v>
+        <v>108</v>
       </c>
       <c r="K20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L20">
         <v>9</v>
@@ -1514,14 +1498,8 @@
       <c r="H21" t="s">
         <v>41</v>
       </c>
-      <c r="I21" t="s">
-        <v>63</v>
-      </c>
-      <c r="J21" t="s">
-        <v>64</v>
-      </c>
       <c r="K21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L21">
         <v>10</v>
@@ -1549,14 +1527,8 @@
       <c r="H22" t="s">
         <v>41</v>
       </c>
-      <c r="I22" t="s">
-        <v>65</v>
-      </c>
-      <c r="J22" t="s">
-        <v>66</v>
-      </c>
       <c r="K22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L22">
         <v>11</v>
@@ -1584,14 +1556,8 @@
       <c r="H23" t="s">
         <v>41</v>
       </c>
-      <c r="I23" t="s">
-        <v>67</v>
-      </c>
-      <c r="J23" t="s">
-        <v>68</v>
-      </c>
       <c r="K23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L23">
         <v>12</v>
@@ -1619,14 +1585,8 @@
       <c r="H24" t="s">
         <v>41</v>
       </c>
-      <c r="I24" t="s">
-        <v>69</v>
-      </c>
-      <c r="J24" t="s">
-        <v>70</v>
-      </c>
       <c r="K24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L24">
         <v>13</v>
@@ -1654,14 +1614,8 @@
       <c r="H25" t="s">
         <v>41</v>
       </c>
-      <c r="I25" t="s">
-        <v>71</v>
-      </c>
-      <c r="J25" t="s">
-        <v>72</v>
-      </c>
       <c r="K25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L25">
         <v>14</v>
@@ -1689,14 +1643,8 @@
       <c r="H26" t="s">
         <v>41</v>
       </c>
-      <c r="I26" t="s">
-        <v>73</v>
-      </c>
-      <c r="J26" t="s">
-        <v>74</v>
-      </c>
       <c r="K26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L26">
         <v>15</v>
@@ -1719,19 +1667,19 @@
         <v>4</v>
       </c>
       <c r="G27" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H27" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I27" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="J27" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="K27" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -1754,19 +1702,19 @@
         <v>4</v>
       </c>
       <c r="G28" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H28" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I28" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="J28" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="K28" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L28">
         <v>1</v>
@@ -1789,19 +1737,19 @@
         <v>4</v>
       </c>
       <c r="G29" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H29" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I29" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="J29" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="K29" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L29">
         <v>2</v>
@@ -1824,19 +1772,19 @@
         <v>4</v>
       </c>
       <c r="G30" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H30" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I30" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="J30" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="K30" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L30">
         <v>3</v>
@@ -1859,19 +1807,19 @@
         <v>4</v>
       </c>
       <c r="G31" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H31" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I31" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="J31" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="K31" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L31">
         <v>4</v>
@@ -1894,19 +1842,19 @@
         <v>4</v>
       </c>
       <c r="G32" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H32" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I32" t="s">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="J32" t="s">
-        <v>89</v>
+        <v>53</v>
       </c>
       <c r="K32" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -1929,19 +1877,19 @@
         <v>4</v>
       </c>
       <c r="G33" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H33" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I33" t="s">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="J33" t="s">
-        <v>91</v>
+        <v>55</v>
       </c>
       <c r="K33" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L33">
         <v>6</v>
@@ -1964,19 +1912,19 @@
         <v>4</v>
       </c>
       <c r="G34" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H34" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I34" t="s">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="J34" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="K34" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L34">
         <v>7</v>
@@ -1999,19 +1947,19 @@
         <v>4</v>
       </c>
       <c r="G35" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H35" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I35" t="s">
-        <v>94</v>
+        <v>58</v>
       </c>
       <c r="J35" t="s">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="K35" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L35">
         <v>8</v>
@@ -2034,19 +1982,19 @@
         <v>4</v>
       </c>
       <c r="G36" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H36" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I36" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="J36" t="s">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="K36" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L36">
         <v>9</v>
@@ -2069,19 +2017,19 @@
         <v>4</v>
       </c>
       <c r="G37" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H37" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I37" t="s">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="J37" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="K37" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L37">
         <v>10</v>
@@ -2104,19 +2052,19 @@
         <v>4</v>
       </c>
       <c r="G38" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H38" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I38" t="s">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="J38" t="s">
-        <v>101</v>
+        <v>65</v>
       </c>
       <c r="K38" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L38">
         <v>11</v>
@@ -2139,19 +2087,19 @@
         <v>4</v>
       </c>
       <c r="G39" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H39" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I39" t="s">
-        <v>102</v>
+        <v>66</v>
       </c>
       <c r="J39" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="K39" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L39">
         <v>12</v>
@@ -2174,19 +2122,19 @@
         <v>4</v>
       </c>
       <c r="G40" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H40" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I40" t="s">
-        <v>104</v>
+        <v>68</v>
       </c>
       <c r="J40" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="K40" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L40">
         <v>13</v>
@@ -2209,19 +2157,19 @@
         <v>4</v>
       </c>
       <c r="G41" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H41" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I41" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="J41" t="s">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="K41" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L41">
         <v>14</v>
@@ -2244,19 +2192,19 @@
         <v>4</v>
       </c>
       <c r="G42" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="H42" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="I42" t="s">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="J42" t="s">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="K42" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="L42">
         <v>15</v>
@@ -2279,10 +2227,10 @@
         <v>5</v>
       </c>
       <c r="G43" t="s">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="H43" t="s">
-        <v>111</v>
+        <v>75</v>
       </c>
       <c r="I43" t="s">
         <v>17</v>
@@ -2299,14 +2247,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
@@ -2314,7 +2262,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -2325,7 +2273,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2333,7 +2281,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2341,7 +2289,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2349,7 +2297,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2357,7 +2305,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2365,7 +2313,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2373,7 +2321,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2381,7 +2329,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2389,7 +2337,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2397,7 +2345,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2405,11 +2353,17 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9d258917-277f-42cd-a3cd-14c4e9ee58bc}" enabled="1" method="Standard" siteId="{38ae3bcd-9579-4fd4-adda-b42e1495d55a}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>